<commit_message>
add func_obj and dummy data
</commit_message>
<xml_diff>
--- a/Instancias Excel/datos.xlsx
+++ b/Instancias Excel/datos.xlsx
@@ -325,19 +325,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>-0.1</v>
+        <v>50000000</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>-1</v>
+        <v>500000</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-100</v>
+        <v>10</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>-1000</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -345,19 +345,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>-0.2</v>
+        <v>100000000</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>-2</v>
+        <v>1000000</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-200</v>
+        <v>20</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>-2000</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -398,19 +398,19 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
-        <v>-1</v>
+        <v>100000</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>-2</v>
+        <v>0.07</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>-3</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1" t="n">
-        <v>-4</v>
+        <v>500000</v>
       </c>
       <c r="E2" s="1" t="n">
-        <v>-5</v>
+        <v>500000</v>
       </c>
     </row>
   </sheetData>
@@ -445,7 +445,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>-10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -453,7 +453,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>-20</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -472,7 +472,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -494,7 +494,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="n">
-        <v>-11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -505,7 +505,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="n">
-        <v>-12</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -516,7 +516,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>-21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -527,7 +527,51 @@
         <v>2</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>-22</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -562,7 +606,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>-10</v>
+        <v>2000000</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -570,7 +614,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>-20</v>
+        <v>3000000</v>
       </c>
     </row>
   </sheetData>
@@ -589,7 +633,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -610,8 +654,8 @@
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="n">
-        <v>-11</v>
+      <c r="C2" s="2" t="n">
+        <v>50000</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -621,8 +665,8 @@
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="n">
-        <v>-12</v>
+      <c r="C3" s="2" t="n">
+        <v>100000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -632,8 +676,8 @@
       <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="1" t="n">
-        <v>-21</v>
+      <c r="C4" s="2" t="n">
+        <v>100000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -643,8 +687,52 @@
       <c r="B5" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>-22</v>
+      <c r="C5" s="2" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2000000</v>
       </c>
     </row>
   </sheetData>
@@ -663,7 +751,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -679,7 +767,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>-10</v>
+        <v>10000000000</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -687,7 +775,23 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>-20</v>
+        <v>10000000000</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>10000000000</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>10000000000</v>
       </c>
     </row>
   </sheetData>
@@ -706,7 +810,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -727,8 +831,8 @@
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="n">
-        <v>-11</v>
+      <c r="C2" s="2" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -738,8 +842,8 @@
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="n">
-        <v>-12</v>
+      <c r="C3" s="2" t="n">
+        <v>100000</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -749,8 +853,8 @@
       <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C4" s="1" t="n">
-        <v>-21</v>
+      <c r="C4" s="2" t="n">
+        <v>100000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -760,8 +864,52 @@
       <c r="B5" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C5" s="1" t="n">
-        <v>-22</v>
+      <c r="C5" s="2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>